<commit_message>
update data after cleaning drive
</commit_message>
<xml_diff>
--- a/Reports/Attendance_Report.xlsx
+++ b/Reports/Attendance_Report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,12 +479,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Aman Kumar</t>
+          <t>Akeel Khan</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ak8102347910@gmail.com</t>
+          <t>akeelkhan3499@gmail.com</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -500,390 +500,390 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mohammad Akeel</t>
+          <t>Akash Kumar Yadav</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>akeelkhan3499@gmail.com</t>
+          <t>akyadav5769@gmail.com</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
         <v>7</v>
       </c>
       <c r="E4" t="n">
-        <v>14.29</v>
+        <v>28.57</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Akash Kumar Yadav</t>
+          <t>Alok</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>akyadav5769@gmail.com</t>
+          <t>alok_kumar@liet.in</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
         <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>28.57</v>
+        <v>14.29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALOK </t>
+          <t xml:space="preserve">Aman Kumar </t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>alok_kumar@liet.in</t>
+          <t>amankumarbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
         <v>7</v>
       </c>
       <c r="E6" t="n">
-        <v>14.29</v>
+        <v>28.57</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Aman Kumar</t>
+          <t xml:space="preserve">Aman Singh </t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>amankumarbtech23-27@liet.in</t>
+          <t>amans64788@gmail.com</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
         <v>7</v>
       </c>
       <c r="E7" t="n">
-        <v>42.86</v>
+        <v>28.57</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Aman Singh</t>
+          <t>Aman singh</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>amans64788@gmail.com</t>
+          <t>amansingh1btech23-27@liet.in</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D8" t="n">
         <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>28.57</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Aman Singh</t>
+          <t xml:space="preserve">Amrendra Ram Tripathi </t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>amansingh1btech23-27@liet.in</t>
+          <t>amrendraramtripathibtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
         <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>85.70999999999999</v>
+        <v>28.57</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Amrendra Ram Tripathi</t>
+          <t>Anshu Gupta</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>amrendraramtripathibtech23-27@liet.in</t>
+          <t>ansh.gup067@gmail.com</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>28.57</v>
+        <v>42.86</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Anshu Gupta</t>
+          <t xml:space="preserve">Ansh Tyagi </t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ansh.gup067@gmail.com</t>
+          <t>anshtyagi189@gmail.com</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D11" t="n">
         <v>7</v>
       </c>
       <c r="E11" t="n">
-        <v>42.86</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Ansh Tyagi</t>
+          <t>Anushka Garg</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>anshtyagi189@gmail.com</t>
+          <t>anushkagargbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D12" t="n">
         <v>7</v>
       </c>
       <c r="E12" t="n">
-        <v>85.70999999999999</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Anushka Garg</t>
+          <t>Anurag Kumar Singh</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>anushkagargbtech23-27@liet.in</t>
+          <t>anusingh99361634@gmail.com</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
         <v>7</v>
       </c>
       <c r="E13" t="n">
-        <v>57.14</v>
+        <v>42.86</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Anurag Kumar Singh</t>
+          <t>Ayush Pal</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>anusingh99361634@gmail.com</t>
+          <t>ayushpalbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
         <v>7</v>
       </c>
       <c r="E14" t="n">
-        <v>42.86</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Ayush Pal</t>
+          <t>Ayush Saw</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ayushpalbtech23-27@liet.in</t>
+          <t>ayushsawbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
         <v>7</v>
       </c>
       <c r="E15" t="n">
-        <v>57.14</v>
+        <v>71.43000000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ayush Saw</t>
+          <t>Ayush Singh</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ayushsawbtech23-27@liet.in</t>
+          <t>ayushsingh50593@gmail.com</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
         <v>7</v>
       </c>
       <c r="E16" t="n">
-        <v>71.43000000000001</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ayush Singh</t>
+          <t>Chetan Goswami</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ayushsingh50593@gmail.com</t>
+          <t>chetangoswami2006@gmail.com</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D17" t="n">
         <v>7</v>
       </c>
       <c r="E17" t="n">
-        <v>57.14</v>
+        <v>71.43000000000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>chetan gooswami</t>
+          <t>Deepanshu</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>chetangoswami2006@gmail.com</t>
+          <t>deepanshu3btech23-27@liet.in</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
         <v>7</v>
       </c>
       <c r="E18" t="n">
-        <v>14.29</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Chetan Goswami</t>
+          <t>Devashish Dobhal</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>chetangoswamibtech23-27@liet.in</t>
+          <t>devashishdobhalbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D19" t="n">
         <v>7</v>
       </c>
       <c r="E19" t="n">
-        <v>57.14</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Deepanshu</t>
+          <t>Garima Singh</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>deepanshu3btech23-27@liet.in</t>
+          <t>gsinghakca@gmail.com</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
         <v>7</v>
       </c>
       <c r="E20" t="n">
-        <v>57.14</v>
+        <v>42.86</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Devashish Dobhal</t>
+          <t xml:space="preserve">Gunjan </t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>devashishdobhalbtech23-27@liet.in</t>
+          <t>gunjanbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D21" t="n">
         <v>7</v>
       </c>
       <c r="E21" t="n">
-        <v>85.70999999999999</v>
+        <v>71.43000000000001</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Garima Singh</t>
+          <t xml:space="preserve">Gurmeet Singh </t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>gsinghakca@gmail.com</t>
+          <t>gurmeetsinghbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -899,54 +899,54 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gunjan</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>gunjanbtech23-27@liet.in</t>
+          <t>happybtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D23" t="n">
         <v>7</v>
       </c>
       <c r="E23" t="n">
-        <v>42.86</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gunjan </t>
+          <t xml:space="preserve">Harshit Rai </t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>gunjanchaudhary@liet.in</t>
+          <t>harshitraibtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D24" t="n">
         <v>7</v>
       </c>
       <c r="E24" t="n">
-        <v>28.57</v>
+        <v>71.43000000000001</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Gurmeet Singh</t>
+          <t>Jai Vardhan Singh</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>gurmeetsinghbtech23-27@liet.in</t>
+          <t>jaisingh1256301@gmail.com</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -962,96 +962,96 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t xml:space="preserve">Kanak Gupta </t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>happybtech23-27@liet.in</t>
+          <t>kanak.gup1234@gmail.com</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D26" t="n">
         <v>7</v>
       </c>
       <c r="E26" t="n">
-        <v>85.70999999999999</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Harshit Rai</t>
+          <t xml:space="preserve">Krishna Kumar Sah </t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>harshitrai1822@gmail.com</t>
+          <t>ksah9189@gmail.com</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>71.43000000000001</v>
+        <v>42.86</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jagat Kumar</t>
+          <t>Ritik</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>jagat.kumar@liet.in</t>
+          <t>kumarritik38269@gmail.com</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D28" t="n">
         <v>7</v>
       </c>
       <c r="E28" t="n">
-        <v>42.86</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Jai</t>
+          <t>Kapil Yadav</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>jaisingh1256301@gmail.com</t>
+          <t>ky205426@gmail.com</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D29" t="n">
         <v>7</v>
       </c>
       <c r="E29" t="n">
-        <v>14.29</v>
+        <v>71.43000000000001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Jai Vardhan Singh</t>
+          <t xml:space="preserve">Manish Mishra </t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>jaivardhansinghbtech23-27@liet.in</t>
+          <t>manishjitendramishrabtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1067,75 +1067,75 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Kanak Gupta</t>
+          <t>Akeel khan</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>kanak.gup1234@gmail.com</t>
+          <t>mohammadakeelbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
         <v>7</v>
       </c>
       <c r="E31" t="n">
-        <v>100</v>
+        <v>14.29</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Krishna Kumar Sah</t>
+          <t>MOHIT</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>krishnakumarsahbtech23-27@liet.in</t>
+          <t>mohitbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D32" t="n">
         <v>7</v>
       </c>
       <c r="E32" t="n">
-        <v>42.86</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ritik</t>
+          <t xml:space="preserve">Mohit Kumar </t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>kumarritik38269@gmail.com</t>
+          <t>mohitkumar746185@gmail.com</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D33" t="n">
         <v>7</v>
       </c>
       <c r="E33" t="n">
-        <v>100</v>
+        <v>28.57</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Kapil Yadav</t>
+          <t xml:space="preserve">Mushroop </t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ky205426@gmail.com</t>
+          <t>mushroopbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1151,12 +1151,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manish Mishra </t>
+          <t xml:space="preserve">Nikhil Sharma </t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>manishjitendramishrabtech23-27@liet.in</t>
+          <t>nikhilsharmabtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1172,285 +1172,285 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>mushroop</t>
+          <t xml:space="preserve">Nilesh Sarkar </t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>mdmushroop@gmail.com</t>
+          <t>nileshsarkar430@email.com</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
         <v>7</v>
       </c>
       <c r="E36" t="n">
-        <v>28.57</v>
+        <v>14.29</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Akeel khan</t>
+          <t xml:space="preserve">Nilesh Sarkar </t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>mohammadakeelbtech23-27@liet.in</t>
+          <t>nileshsarkar430@gmail.com</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D37" t="n">
         <v>7</v>
       </c>
       <c r="E37" t="n">
-        <v>14.29</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mohit</t>
+          <t xml:space="preserve">Nisha Gupta </t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>mohitbtech23-27@liet.in</t>
+          <t>nishaguptabtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D38" t="n">
         <v>7</v>
       </c>
       <c r="E38" t="n">
-        <v>85.70999999999999</v>
+        <v>28.57</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Mohit Kumar</t>
+          <t>PIYUSH SINGH</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>mohitkumar746185@gmail.com</t>
+          <t>piyushsingh1982004@gmail.com</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D39" t="n">
         <v>7</v>
       </c>
       <c r="E39" t="n">
-        <v>28.57</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mushroop </t>
+          <t xml:space="preserve">Prateek Rai </t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>mushroopbtech23-27@liet.in</t>
+          <t>prateekraibtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D40" t="n">
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>14.29</v>
+        <v>71.43000000000001</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>mushroop</t>
+          <t>Prem Kumar Jha</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>mushroopmd08@gmail.com</t>
+          <t>premkumarjhabtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D41" t="n">
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>14.29</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Nilesh Sarkar</t>
+          <t xml:space="preserve">Pushpendra Yadav </t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>nileshsarkar430@gmail.com</t>
+          <t>pushpendrayadav8434@gmail.com</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D42" t="n">
         <v>7</v>
       </c>
       <c r="E42" t="n">
-        <v>100</v>
+        <v>71.43000000000001</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Nisha Gupta</t>
+          <t>Rahul Yadav</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>nishaguptabtech23-27@liet.in</t>
+          <t>rahulyadavbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D43" t="n">
         <v>7</v>
       </c>
       <c r="E43" t="n">
-        <v>28.57</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Nikhil Sharma</t>
+          <t>Ritesh Kumar Singh</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ns977440@gmail.com</t>
+          <t>riteshkumar07.com@gmail.com</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44" t="n">
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>14.29</v>
+        <v>28.57</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Piyush Singh</t>
+          <t xml:space="preserve">Rohit Kumar </t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>piyushsinghbtech23-27@liet.in</t>
+          <t>rohitkumarbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D45" t="n">
         <v>7</v>
       </c>
       <c r="E45" t="n">
-        <v>85.70999999999999</v>
+        <v>71.43000000000001</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Prem Kumar Jha</t>
+          <t>Sakshi Chauhan</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>premkumarjhabtech23-27@liet.in</t>
+          <t>sakshichauhanbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D46" t="n">
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>57.14</v>
+        <v>100</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Pushpendra Yadav</t>
+          <t xml:space="preserve">Sanskar </t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>pushpendrayadav8434@gmail.com</t>
+          <t>sanskarbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D47" t="n">
         <v>7</v>
       </c>
       <c r="E47" t="n">
-        <v>71.43000000000001</v>
+        <v>28.57</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Rahul Yadav</t>
+          <t xml:space="preserve">Satyansh Rawat </t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>rahulyadavbtech23-27@liet.in</t>
+          <t>satyanshrawatbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D48" t="n">
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>57.14</v>
+        <v>71.43000000000001</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Prateek Rai</t>
+          <t xml:space="preserve">Shivam Chaudhary </t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>raiprateek009@gmail.com</t>
+          <t>shivamchaudharybtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1466,33 +1466,33 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ritesh Kumar Singh</t>
+          <t xml:space="preserve">Shivangi Pandey </t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>riteshkumar07.com@gmail.com</t>
+          <t>shivangipandeyabc@gmail.com</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D50" t="n">
         <v>7</v>
       </c>
       <c r="E50" t="n">
-        <v>28.57</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Rohit Kumar</t>
+          <t>Sonu Kumar</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>rohitkumarbtech23-27@liet.in</t>
+          <t>sonukumarbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1508,33 +1508,33 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Sakshi Chauhan</t>
+          <t xml:space="preserve">Sringani Singh </t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>sakshichauhan5997@gmail.com</t>
+          <t>sringanisinghbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D52" t="n">
         <v>7</v>
       </c>
       <c r="E52" t="n">
-        <v>100</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Satyansh Rawat</t>
+          <t>Tarun kumar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>satyanshrawatbtech23-27@liet.in</t>
+          <t>tarunkumar1btech23-27@liet.in</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -1550,54 +1550,54 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Shivam Chaudhary</t>
+          <t>Vaibhav Mishra</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>shivamchaudharybtech23-27@liet.in</t>
+          <t>vaibhavmishrabtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D54" t="n">
         <v>7</v>
       </c>
       <c r="E54" t="n">
-        <v>71.43000000000001</v>
+        <v>42.86</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Shivangi Pandey</t>
+          <t>Vibhu</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>shivangipandeyabc@gmail.com</t>
+          <t>vibhubtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D55" t="n">
         <v>7</v>
       </c>
       <c r="E55" t="n">
-        <v>85.70999999999999</v>
+        <v>14.29</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Sanskar</t>
+          <t>Vineet Kumar Roy</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>solankisanskar01@gmail.com</t>
+          <t>vineet333roy@gmail.com</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -1613,299 +1613,126 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Sonu Kumar</t>
+          <t xml:space="preserve">Vipul Pandey </t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>sonukumar3570357@gmail.com</t>
+          <t>vipulpandeybtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D57" t="n">
         <v>7</v>
       </c>
       <c r="E57" t="n">
-        <v>71.43000000000001</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Sringani Singh</t>
+          <t xml:space="preserve">Vishujeet Rathore </t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>sringanisinghbtech23-27@liet.in</t>
+          <t>vishujeetrathor@gmail.com</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D58" t="n">
         <v>7</v>
       </c>
       <c r="E58" t="n">
-        <v>57.14</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Tarun Kumar</t>
+          <t>Vivek Yadav</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>tarunpandit885@gmail.com</t>
+          <t>vivekyadavbtech23-27@liet.in</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D59" t="n">
         <v>7</v>
       </c>
       <c r="E59" t="n">
-        <v>71.43000000000001</v>
+        <v>100</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Vaibhav Mishra</t>
+          <t>Vishal Kumar</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>vaibhavmishrabtech23-27@liet.in</t>
+          <t>vk9491015@gmail.com</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D60" t="n">
         <v>7</v>
       </c>
       <c r="E60" t="n">
-        <v>42.86</v>
+        <v>71.43000000000001</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Vineet Kumar Roy</t>
+          <t xml:space="preserve">Shreyanshi Yadav </t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>vineet333roy@gmail.com</t>
+          <t>yadavshreyanshi772@gmail.com</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D61" t="n">
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>28.57</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Vipul Pandey</t>
+          <t>Yash Bansal</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>vipulpandeybtech23-27@liet.in</t>
+          <t>yashbansal216@gmail.com</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D62" t="n">
         <v>7</v>
       </c>
       <c r="E62" t="n">
-        <v>85.70999999999999</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Vishujeet Rathore</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>vishujeetrathor@gmail.com</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>5</v>
-      </c>
-      <c r="D63" t="n">
-        <v>7</v>
-      </c>
-      <c r="E63" t="n">
-        <v>71.43000000000001</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Vivek Yadav</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>vivekyadavbtech23-27@liet.in</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>7</v>
-      </c>
-      <c r="D64" t="n">
-        <v>7</v>
-      </c>
-      <c r="E64" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Vishal Kumar</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>vk9491015@gmail.com</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>5</v>
-      </c>
-      <c r="D65" t="n">
-        <v>7</v>
-      </c>
-      <c r="E65" t="n">
-        <v>71.43000000000001</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Shreyanshi Yadav</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>yadavshreyanshi022@gmail.com</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>4</v>
-      </c>
-      <c r="D66" t="n">
-        <v>7</v>
-      </c>
-      <c r="E66" t="n">
-        <v>57.14</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Yash Bansal</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>yashbansal216@gmail.com</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>2</v>
-      </c>
-      <c r="D67" t="n">
-        <v>7</v>
-      </c>
-      <c r="E67" t="n">
-        <v>28.57</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Karan Sharma </t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="n">
-        <v>2</v>
-      </c>
-      <c r="D68" t="n">
-        <v>7</v>
-      </c>
-      <c r="E68" t="n">
-        <v>28.57</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Karan Sharma </t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="n">
-        <v>2</v>
-      </c>
-      <c r="D69" t="n">
-        <v>7</v>
-      </c>
-      <c r="E69" t="n">
-        <v>28.57</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Karan Sharma </t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="n">
-        <v>2</v>
-      </c>
-      <c r="D70" t="n">
-        <v>7</v>
-      </c>
-      <c r="E70" t="n">
-        <v>28.57</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Karan Sharma </t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="n">
-        <v>2</v>
-      </c>
-      <c r="D71" t="n">
-        <v>7</v>
-      </c>
-      <c r="E71" t="n">
         <v>28.57</v>
       </c>
     </row>

</xml_diff>